<commit_message>
update(journalTrav) update pour le journal d'hier
</commit_message>
<xml_diff>
--- a/documentation/JDT-personal/Journal-de-Travail_PiguetAntoine.xlsx
+++ b/documentation/JDT-personal/Journal-de-Travail_PiguetAntoine.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn01kbc\Documents\MODULE T4\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pn01kbc\Documents\GitHub\Passion_lecture_FRONTEND\documentation\JDT-personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4E02A85-AB66-46C2-9924-C47D7C682A1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5D644D6-5E48-474F-AFC4-13D1CB9BFE2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="Mvap2W10CJFFJsnvkGXSiMLvpngxTMJbJsIKFe7Hzjn0XDcmjGuvBC2FjUCZ/hpRpUhUrG1T4kBlDAIo3yqmSQ==" workbookSaltValue="KXjgXOcsUZI/j7UgPKltzw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="39">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -149,6 +149,15 @@
   </si>
   <si>
     <t>J'ai revu et modifié un peu la maquette pour être bien sûr qu'elle corresponde au CdC</t>
+  </si>
+  <si>
+    <t>Avec C-H, on s'est retrouvé face à une erreur spéciale: on avait 2 versions de la route register, une sous le nom de register et une sous le nom de user. On faisait les modifs sur l'ancienne version alors que la route utilisée était celle de la nouvelle. On ne comprenait donc pas pourquoi les changements ne se faisaient pas.</t>
+  </si>
+  <si>
+    <t>J'ai amélioré et rendu fonctionnel la page de register. Maintenant, la page envoie le form au back, le back le mets dans la db si OK et renvoie un token au front qui le met dans localStorage pour qu'il soit accessible depuis tout le code.</t>
+  </si>
+  <si>
+    <t>J'ai aussi modifié le header pour ajouter des boutons login/register et du backend pour bien répondre à nos routes. Ainsi que des modifs dans le back par rapport aux tokens.</t>
   </si>
 </sst>
 </file>
@@ -1079,7 +1088,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.16666666666666666</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2057,7 +2066,7 @@
       </c>
       <c r="C3" s="22" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 5 heurs 30 minutes</v>
+        <v>0 jours 9 heurs 30 minutes</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="3"/>
@@ -2072,7 +2081,7 @@
       <c r="B4" s="5"/>
       <c r="C4" s="22">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>240</v>
+        <v>480</v>
       </c>
       <c r="D4" s="22">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
@@ -2080,7 +2089,7 @@
       </c>
       <c r="E4" s="40">
         <f>SUM(C4:D4)</f>
-        <v>330</v>
+        <v>570</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2329,16 +2338,24 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="16" t="str">
+    <row r="15" spans="1:15" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A15" s="16">
         <f>IF(ISBLANK(B15),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B15))</f>
-        <v/>
-      </c>
-      <c r="B15" s="50"/>
-      <c r="C15" s="51"/>
+        <v>21</v>
+      </c>
+      <c r="B15" s="50">
+        <v>45797</v>
+      </c>
+      <c r="C15" s="51">
+        <v>2</v>
+      </c>
       <c r="D15" s="52"/>
-      <c r="E15" s="53"/>
-      <c r="F15" s="36"/>
+      <c r="E15" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="F15" s="36" t="s">
+        <v>37</v>
+      </c>
       <c r="G15" s="56"/>
       <c r="M15" t="s">
         <v>22</v>
@@ -2350,31 +2367,47 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="str">
+    <row r="16" spans="1:15" ht="63" x14ac:dyDescent="0.25">
+      <c r="A16" s="8">
         <f>IF(ISBLANK(B16),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B16))</f>
-        <v/>
-      </c>
-      <c r="B16" s="46"/>
-      <c r="C16" s="47"/>
+        <v>21</v>
+      </c>
+      <c r="B16" s="46">
+        <v>45797</v>
+      </c>
+      <c r="C16" s="47">
+        <v>1</v>
+      </c>
       <c r="D16" s="48"/>
-      <c r="E16" s="49"/>
-      <c r="F16" s="36"/>
+      <c r="E16" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="F16" s="36" t="s">
+        <v>36</v>
+      </c>
       <c r="G16" s="55"/>
       <c r="O16">
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="str">
+    <row r="17" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="16">
         <f>IF(ISBLANK(B17),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B17))</f>
-        <v/>
-      </c>
-      <c r="B17" s="50"/>
-      <c r="C17" s="51"/>
+        <v>21</v>
+      </c>
+      <c r="B17" s="50">
+        <v>45797</v>
+      </c>
+      <c r="C17" s="51">
+        <v>1</v>
+      </c>
       <c r="D17" s="52"/>
-      <c r="E17" s="53"/>
-      <c r="F17" s="36"/>
+      <c r="E17" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="F17" s="36" t="s">
+        <v>38</v>
+      </c>
       <c r="G17" s="56"/>
       <c r="O17">
         <v>45</v>
@@ -8663,7 +8696,7 @@
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
@@ -8675,7 +8708,7 @@
       </c>
       <c r="D5" s="33">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>0</v>
+        <v>0.16666666666666666</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -8792,7 +8825,7 @@
       </c>
       <c r="D12" s="34">
         <f>SUM(D4:D11)</f>
-        <v>0.22916666666666666</v>
+        <v>0.39583333333333331</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -8815,17 +8848,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D4F20F00DBE2EE49BE9523363A2DF18B" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="313dbdbec26224d1c2bb7e3c488b2a4e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="99ffe1f3-7857-457f-add0-5bdef636f38d" xmlns:ns3="be0d3259-a7ce-4623-88ec-81594dfcbc1c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4739345e3d2c6be79c5ae1a54d02a4a7" ns2:_="" ns3:_="">
     <xsd:import namespace="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
@@ -9048,6 +9070,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="be0d3259-a7ce-4623-88ec-81594dfcbc1c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99ffe1f3-7857-457f-add0-5bdef636f38d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
@@ -9057,17 +9090,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2FB702A-DCBD-43A8-A34C-6000FD8861AD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9084,4 +9106,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>